<commit_message>
Add ADC IFC sweep measurements
</commit_message>
<xml_diff>
--- a/frequency sweep.xlsx
+++ b/frequency sweep.xlsx
@@ -8,29 +8,43 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TIDIAC\summer2025_research_tiadc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C83AA96-BFCB-4076-92DE-3F4E1F607126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794437B8-DE7D-4298-A411-EFD13ED59704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
-    <t>ampl(mV)</t>
+    <t>freq(MHz)</t>
   </si>
   <si>
-    <t>freq(MHz)</t>
+    <t>amplitude (mV)</t>
+  </si>
+  <si>
+    <t>resolution (µV/code)</t>
   </si>
 </sst>
 </file>
@@ -348,183 +362,274 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1.25</v>
       </c>
       <c r="B2">
         <v>100</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2">
+        <f>(B2*0.001)/2^16*1000000</f>
+        <v>1.52587890625</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2.5</v>
       </c>
       <c r="B3">
         <v>163</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3">
+        <f t="shared" ref="C3:C22" si="0">(B3*0.001)/2^16*1000000</f>
+        <v>2.4871826171875</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>5</v>
       </c>
       <c r="B4">
         <v>330</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>5.035400390625</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>7.5</v>
       </c>
       <c r="B5">
         <v>450</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>6.866455078125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>10</v>
       </c>
       <c r="B6">
         <v>533</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>8.1329345703125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>12.5</v>
       </c>
       <c r="B7">
         <v>600</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>9.1552734375</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>15</v>
       </c>
       <c r="B8">
         <v>652</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>9.94873046875</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>20</v>
       </c>
       <c r="B9">
         <v>720</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>10.986328125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>25</v>
       </c>
       <c r="B10">
         <v>764</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>11.65771484375</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>35</v>
       </c>
       <c r="B11">
         <v>830</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>12.664794921875002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>50</v>
       </c>
       <c r="B12">
         <v>870</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>13.275146484375</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>75</v>
       </c>
       <c r="B13">
         <v>915</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>13.9617919921875</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>100</v>
       </c>
       <c r="B14">
         <v>950</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C14">
+        <f t="shared" si="0"/>
+        <v>14.495849609375002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>200</v>
       </c>
       <c r="B15">
         <v>969</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>14.7857666015625</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>300</v>
       </c>
       <c r="B16">
         <v>875</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>13.3514404296875</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>400</v>
       </c>
       <c r="B17">
         <v>979</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <f t="shared" si="0"/>
+        <v>14.9383544921875</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>500</v>
       </c>
       <c r="B18">
         <v>875</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18">
+        <f t="shared" si="0"/>
+        <v>13.3514404296875</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>625</v>
       </c>
       <c r="B19">
         <v>916</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19">
+        <f t="shared" si="0"/>
+        <v>13.97705078125</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>750</v>
       </c>
       <c r="B20">
         <v>778</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20">
+        <f t="shared" si="0"/>
+        <v>11.871337890625</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1000</v>
       </c>
       <c r="B21">
         <v>755</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21">
+        <f t="shared" si="0"/>
+        <v>11.5203857421875</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1200</v>
       </c>
       <c r="B22">
         <v>628</v>
+      </c>
+      <c r="C22">
+        <f t="shared" si="0"/>
+        <v>9.58251953125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>